<commit_message>
i have added more
</commit_message>
<xml_diff>
--- a/farmers_analysis.xlsx
+++ b/farmers_analysis.xlsx
@@ -50,12 +50,6 @@
     <t>Credit Access</t>
   </si>
   <si>
-    <t>Yield Before (kg/ha)</t>
-  </si>
-  <si>
-    <t>Yield After (kg/ha)</t>
-  </si>
-  <si>
     <t>Training Attended</t>
   </si>
   <si>
@@ -249,6 +243,12 @@
   </si>
   <si>
     <t>Farm Size ha</t>
+  </si>
+  <si>
+    <t>Yield Before kg per hec</t>
+  </si>
+  <si>
+    <t>Yield Change</t>
   </si>
 </sst>
 </file>
@@ -675,7 +675,7 @@
     <col min="7" max="7" width="17.1796875" customWidth="1"/>
     <col min="8" max="8" width="14.81640625" customWidth="1"/>
     <col min="9" max="9" width="15.26953125" customWidth="1"/>
-    <col min="10" max="10" width="21.54296875" customWidth="1"/>
+    <col min="10" max="10" width="24.36328125" customWidth="1"/>
     <col min="11" max="11" width="23.54296875" customWidth="1"/>
     <col min="12" max="12" width="21.54296875" customWidth="1"/>
     <col min="13" max="13" width="20.81640625" customWidth="1"/>
@@ -709,10 +709,10 @@
         <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>4</v>
@@ -727,27 +727,27 @@
         <v>7</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D3" s="2">
         <v>0.9</v>
@@ -756,16 +756,16 @@
         <v>76.099999999999994</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J3" s="2">
         <v>6714</v>
@@ -777,18 +777,18 @@
         <v>15.6</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D4" s="5">
         <v>0.6</v>
@@ -797,16 +797,16 @@
         <v>41.4</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J4" s="5">
         <v>4753</v>
@@ -818,18 +818,18 @@
         <v>13.8</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="2">
         <v>1</v>
@@ -838,16 +838,16 @@
         <v>47.8</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J5" s="2">
         <v>4679</v>
@@ -859,18 +859,18 @@
         <v>20.8</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" s="5">
         <v>2.7</v>
@@ -879,16 +879,16 @@
         <v>38.200000000000003</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J6" s="5">
         <v>5892</v>
@@ -900,18 +900,18 @@
         <v>15.6</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D7" s="2">
         <v>1.2</v>
@@ -920,16 +920,16 @@
         <v>31.6</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J7" s="2">
         <v>6857</v>
@@ -941,18 +941,18 @@
         <v>18.3</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D8" s="5">
         <v>2</v>
@@ -961,16 +961,16 @@
         <v>74.2</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J8" s="5">
         <v>5362</v>
@@ -982,18 +982,18 @@
         <v>15</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D9" s="2">
         <v>3.2</v>
@@ -1002,16 +1002,16 @@
         <v>50</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J9" s="2">
         <v>4727</v>
@@ -1023,18 +1023,18 @@
         <v>14</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D10" s="5">
         <v>1</v>
@@ -1043,16 +1043,16 @@
         <v>64</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J10" s="5">
         <v>5670</v>
@@ -1064,18 +1064,18 @@
         <v>13.8</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D11" s="2">
         <v>2.5</v>
@@ -1084,16 +1084,16 @@
         <v>35.700000000000003</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J11" s="2">
         <v>5350</v>
@@ -1105,18 +1105,18 @@
         <v>18.8</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D12" s="5">
         <v>1.9</v>
@@ -1125,16 +1125,16 @@
         <v>77.7</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J12" s="5">
         <v>4947</v>
@@ -1146,18 +1146,18 @@
         <v>22.5</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D13" s="2">
         <v>1.4</v>
@@ -1166,16 +1166,16 @@
         <v>61.9</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J13" s="2">
         <v>4848</v>
@@ -1187,18 +1187,18 @@
         <v>17.100000000000001</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D14" s="5">
         <v>2.2999999999999998</v>
@@ -1207,16 +1207,16 @@
         <v>54.4</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J14" s="5">
         <v>6517</v>
@@ -1228,18 +1228,18 @@
         <v>14.7</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D15" s="2">
         <v>3.3</v>
@@ -1248,16 +1248,16 @@
         <v>34.299999999999997</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J15" s="2">
         <v>6415</v>
@@ -1269,18 +1269,18 @@
         <v>13.3</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D16" s="5">
         <v>1</v>
@@ -1289,16 +1289,16 @@
         <v>56.4</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J16" s="5">
         <v>6388</v>
@@ -1310,18 +1310,18 @@
         <v>16</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D17" s="2">
         <v>3.5</v>
@@ -1330,16 +1330,16 @@
         <v>62.5</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J17" s="2">
         <v>4062</v>
@@ -1351,18 +1351,18 @@
         <v>14.3</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D18" s="5">
         <v>2.2999999999999998</v>
@@ -1371,16 +1371,16 @@
         <v>30.4</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J18" s="5">
         <v>3579</v>
@@ -1392,18 +1392,18 @@
         <v>19</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D19" s="2">
         <v>1.2</v>
@@ -1412,16 +1412,16 @@
         <v>63.4</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J19" s="2">
         <v>5928</v>
@@ -1433,18 +1433,18 @@
         <v>14.5</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D20" s="5">
         <v>1.1000000000000001</v>
@@ -1453,16 +1453,16 @@
         <v>34.799999999999997</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J20" s="5">
         <v>6323</v>
@@ -1474,18 +1474,18 @@
         <v>15.1</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D21" s="2">
         <v>0.7</v>
@@ -1494,16 +1494,16 @@
         <v>66.400000000000006</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J21" s="2">
         <v>4841</v>
@@ -1515,18 +1515,18 @@
         <v>17.8</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D22" s="5">
         <v>1.3</v>
@@ -1535,16 +1535,16 @@
         <v>42.5</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J22" s="5">
         <v>5876</v>
@@ -1556,18 +1556,18 @@
         <v>17.3</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D23" s="2">
         <v>3</v>
@@ -1576,16 +1576,16 @@
         <v>78.400000000000006</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J23" s="2">
         <v>4714</v>
@@ -1597,18 +1597,18 @@
         <v>18.3</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D24" s="5">
         <v>3.2</v>
@@ -1617,16 +1617,16 @@
         <v>38.200000000000003</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J24" s="5">
         <v>6463</v>
@@ -1638,18 +1638,18 @@
         <v>13.6</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D25" s="2">
         <v>3.5</v>
@@ -1658,16 +1658,16 @@
         <v>57.8</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J25" s="2">
         <v>5922</v>
@@ -1679,18 +1679,18 @@
         <v>20.5</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D26" s="5">
         <v>0.7</v>
@@ -1699,16 +1699,16 @@
         <v>45.7</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J26" s="5">
         <v>4828</v>
@@ -1720,18 +1720,18 @@
         <v>12.8</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D27" s="2">
         <v>0.7</v>
@@ -1740,16 +1740,16 @@
         <v>33.4</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J27" s="2">
         <v>4924</v>
@@ -1761,18 +1761,18 @@
         <v>20.5</v>
       </c>
       <c r="M27" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D28" s="5">
         <v>2.4</v>
@@ -1781,16 +1781,16 @@
         <v>51</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J28" s="5">
         <v>4011</v>
@@ -1802,18 +1802,18 @@
         <v>17.600000000000001</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D29" s="2">
         <v>0.9</v>
@@ -1822,16 +1822,16 @@
         <v>62.3</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J29" s="2">
         <v>4523</v>
@@ -1843,18 +1843,18 @@
         <v>16</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D30" s="5">
         <v>0.7</v>
@@ -1863,16 +1863,16 @@
         <v>40.700000000000003</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J30" s="5">
         <v>6698</v>
@@ -1884,18 +1884,18 @@
         <v>15.8</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D31" s="2">
         <v>2.6</v>
@@ -1904,16 +1904,16 @@
         <v>60.6</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J31" s="2">
         <v>6543</v>
@@ -1925,18 +1925,18 @@
         <v>18.8</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D32" s="5">
         <v>0.8</v>
@@ -1945,16 +1945,16 @@
         <v>73.900000000000006</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J32" s="5">
         <v>3889</v>
@@ -1966,18 +1966,18 @@
         <v>15.1</v>
       </c>
       <c r="M32" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D33" s="2">
         <v>1.1000000000000001</v>
@@ -1986,16 +1986,16 @@
         <v>25.9</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J33" s="2">
         <v>5615</v>
@@ -2007,18 +2007,18 @@
         <v>-3.8</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D34" s="5">
         <v>0.6</v>
@@ -2027,16 +2027,16 @@
         <v>18.3</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J34" s="5">
         <v>4605</v>
@@ -2048,18 +2048,18 @@
         <v>-1.2</v>
       </c>
       <c r="M34" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D35" s="2">
         <v>0.7</v>
@@ -2068,16 +2068,16 @@
         <v>32.1</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J35" s="2">
         <v>4956</v>
@@ -2089,18 +2089,18 @@
         <v>0.7</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D36" s="5">
         <v>0.6</v>
@@ -2109,16 +2109,16 @@
         <v>19.100000000000001</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J36" s="5">
         <v>4395</v>
@@ -2130,18 +2130,18 @@
         <v>3.4</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D37" s="2">
         <v>0.8</v>
@@ -2150,16 +2150,16 @@
         <v>29.5</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J37" s="2">
         <v>4886</v>
@@ -2171,18 +2171,18 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="M37" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D38" s="5">
         <v>3.4</v>
@@ -2191,16 +2191,16 @@
         <v>30.3</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J38" s="5">
         <v>4330</v>
@@ -2212,18 +2212,18 @@
         <v>4.7</v>
       </c>
       <c r="M38" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D39" s="2">
         <v>3.1</v>
@@ -2232,16 +2232,16 @@
         <v>30.3</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J39" s="2">
         <v>5680</v>
@@ -2253,18 +2253,18 @@
         <v>0.6</v>
       </c>
       <c r="M39" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D40" s="5">
         <v>1.5</v>
@@ -2273,16 +2273,16 @@
         <v>30.5</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J40" s="5">
         <v>5496</v>
@@ -2294,18 +2294,18 @@
         <v>1.4</v>
       </c>
       <c r="M40" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D41" s="2">
         <v>3.4</v>
@@ -2314,16 +2314,16 @@
         <v>17</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J41" s="2">
         <v>5841</v>
@@ -2335,18 +2335,18 @@
         <v>1.4</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D42" s="5">
         <v>1</v>
@@ -2355,16 +2355,16 @@
         <v>34.1</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I42" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J42" s="5">
         <v>5321</v>
@@ -2376,18 +2376,18 @@
         <v>-3.3</v>
       </c>
       <c r="M42" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D43" s="2">
         <v>0.8</v>
@@ -2396,16 +2396,16 @@
         <v>32.5</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J43" s="2">
         <v>5800</v>
@@ -2417,18 +2417,18 @@
         <v>-1</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D44" s="5">
         <v>2.7</v>
@@ -2437,16 +2437,16 @@
         <v>14.9</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J44" s="5">
         <v>5058</v>
@@ -2458,18 +2458,18 @@
         <v>-0.1</v>
       </c>
       <c r="M44" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D45" s="2">
         <v>2</v>
@@ -2478,16 +2478,16 @@
         <v>26.7</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J45" s="2">
         <v>4980</v>
@@ -2499,18 +2499,18 @@
         <v>-0.8</v>
       </c>
       <c r="M45" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D46" s="5">
         <v>3.2</v>
@@ -2519,16 +2519,16 @@
         <v>25.4</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J46" s="5">
         <v>5217</v>
@@ -2540,18 +2540,18 @@
         <v>-2.6</v>
       </c>
       <c r="M46" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D47" s="2">
         <v>1.5</v>
@@ -2560,16 +2560,16 @@
         <v>21</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J47" s="2">
         <v>6900</v>
@@ -2581,18 +2581,18 @@
         <v>3.7</v>
       </c>
       <c r="M47" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D48" s="5">
         <v>0.8</v>
@@ -2601,16 +2601,16 @@
         <v>22.9</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J48" s="5">
         <v>6378</v>
@@ -2622,18 +2622,18 @@
         <v>-0.3</v>
       </c>
       <c r="M48" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D49" s="2">
         <v>0.9</v>
@@ -2642,16 +2642,16 @@
         <v>11.2</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J49" s="2">
         <v>5639</v>
@@ -2663,18 +2663,18 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="M49" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D50" s="5">
         <v>1.1000000000000001</v>
@@ -2683,16 +2683,16 @@
         <v>27.4</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J50" s="5">
         <v>4514</v>
@@ -2704,18 +2704,18 @@
         <v>-1.6</v>
       </c>
       <c r="M50" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D51" s="2">
         <v>2.8</v>
@@ -2724,16 +2724,16 @@
         <v>15.5</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J51" s="2">
         <v>5894</v>
@@ -2745,18 +2745,18 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A52" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D52" s="5">
         <v>1.9</v>
@@ -2765,16 +2765,16 @@
         <v>30</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G52" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J52" s="5">
         <v>5875</v>
@@ -2786,7 +2786,7 @@
         <v>4.5</v>
       </c>
       <c r="M52" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>